<commit_message>
Universum Stand 09.10.: EA, WBD, AVB inaktiv; PSKY → SKYD, EQR → VMRK (SQL, Excel, MANUAL_OVERRIDES leer)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/universum-pruefung.xlsx
+++ b/docs/universum-pruefung.xlsx
@@ -1,12 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10916"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B12583E-67AF-AE47-A7CD-2FF144C65060}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Universum" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Legende" state="visible" r:id="rId5"/>
+    <sheet name="Universum" sheetId="1" r:id="rId1"/>
+    <sheet name="Legende" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Universum!$A$1:$Q$505</definedName>
+  </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
@@ -6449,17 +6456,20 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -6537,7 +6547,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -6873,9 +6883,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q505"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="34" customWidth="1"/>
     <col min="3" max="3" width="12" style="1" customWidth="1"/>
@@ -6894,7 +6904,7 @@
     <col min="17" max="17" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -6947,7 +6957,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>17</v>
       </c>
@@ -7000,7 +7010,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>28</v>
       </c>
@@ -7053,7 +7063,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>35</v>
       </c>
@@ -7106,7 +7116,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>38</v>
       </c>
@@ -7159,7 +7169,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>44</v>
       </c>
@@ -7212,7 +7222,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>50</v>
       </c>
@@ -7265,7 +7275,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>53</v>
       </c>
@@ -7318,7 +7328,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>59</v>
       </c>
@@ -7371,7 +7381,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>62</v>
       </c>
@@ -7424,7 +7434,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>65</v>
       </c>
@@ -7477,7 +7487,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>72</v>
       </c>
@@ -7530,7 +7540,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
         <v>79</v>
       </c>
@@ -7583,7 +7593,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
         <v>86</v>
       </c>
@@ -7636,7 +7646,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
         <v>92</v>
       </c>
@@ -7689,7 +7699,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
         <v>95</v>
       </c>
@@ -7742,7 +7752,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
         <v>98</v>
       </c>
@@ -7795,7 +7805,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
         <v>101</v>
       </c>
@@ -7848,7 +7858,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
         <v>104</v>
       </c>
@@ -7901,7 +7911,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
         <v>107</v>
       </c>
@@ -7954,7 +7964,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
         <v>113</v>
       </c>
@@ -8007,7 +8017,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
         <v>116</v>
       </c>
@@ -8060,7 +8070,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
         <v>119</v>
       </c>
@@ -8113,7 +8123,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
         <v>122</v>
       </c>
@@ -8166,7 +8176,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
         <v>125</v>
       </c>
@@ -8219,7 +8229,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
         <v>128</v>
       </c>
@@ -8272,7 +8282,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
         <v>131</v>
       </c>
@@ -8325,7 +8335,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
         <v>134</v>
       </c>
@@ -8378,7 +8388,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:17" ht="64" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
         <v>140</v>
       </c>
@@ -8431,7 +8441,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
         <v>146</v>
       </c>
@@ -8484,7 +8494,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
         <v>149</v>
       </c>
@@ -8537,7 +8547,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
         <v>152</v>
       </c>
@@ -8590,7 +8600,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:17" ht="64" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
         <v>155</v>
       </c>
@@ -8643,7 +8653,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
         <v>158</v>
       </c>
@@ -8696,7 +8706,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
         <v>161</v>
       </c>
@@ -8749,7 +8759,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
         <v>164</v>
       </c>
@@ -8802,7 +8812,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
         <v>167</v>
       </c>
@@ -8855,7 +8865,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
         <v>170</v>
       </c>
@@ -8908,7 +8918,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
         <v>177</v>
       </c>
@@ -8961,7 +8971,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="s">
         <v>180</v>
       </c>
@@ -9014,7 +9024,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
         <v>183</v>
       </c>
@@ -9067,7 +9077,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
         <v>190</v>
       </c>
@@ -9120,7 +9130,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:17" ht="64" x14ac:dyDescent="0.2">
       <c r="A43" s="5" t="s">
         <v>193</v>
       </c>
@@ -9173,7 +9183,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A44" s="5" t="s">
         <v>196</v>
       </c>
@@ -9226,7 +9236,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A45" s="5" t="s">
         <v>199</v>
       </c>
@@ -9279,7 +9289,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A46" s="5" t="s">
         <v>202</v>
       </c>
@@ -9332,7 +9342,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A47" s="5" t="s">
         <v>205</v>
       </c>
@@ -9385,7 +9395,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" s="5" t="s">
         <v>208</v>
       </c>
@@ -9438,7 +9448,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A49" s="5" t="s">
         <v>211</v>
       </c>
@@ -9491,7 +9501,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A50" s="5" t="s">
         <v>214</v>
       </c>
@@ -9544,7 +9554,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A51" s="5" t="s">
         <v>217</v>
       </c>
@@ -9597,7 +9607,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:17" ht="64" x14ac:dyDescent="0.2">
       <c r="A52" s="5" t="s">
         <v>220</v>
       </c>
@@ -9650,7 +9660,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:17" ht="64" x14ac:dyDescent="0.2">
       <c r="A53" s="5" t="s">
         <v>223</v>
       </c>
@@ -9703,7 +9713,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A54" s="5" t="s">
         <v>226</v>
       </c>
@@ -9756,7 +9766,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A55" s="5" t="s">
         <v>229</v>
       </c>
@@ -9809,7 +9819,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" s="5" t="s">
         <v>232</v>
       </c>
@@ -9862,7 +9872,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A57" s="5" t="s">
         <v>238</v>
       </c>
@@ -9915,7 +9925,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A58" s="5" t="s">
         <v>241</v>
       </c>
@@ -9968,7 +9978,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A59" s="5" t="s">
         <v>244</v>
       </c>
@@ -10021,7 +10031,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A60" s="5" t="s">
         <v>247</v>
       </c>
@@ -10074,7 +10084,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A61" s="5" t="s">
         <v>250</v>
       </c>
@@ -10127,7 +10137,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A62" s="5" t="s">
         <v>253</v>
       </c>
@@ -10180,7 +10190,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A63" s="5" t="s">
         <v>256</v>
       </c>
@@ -10233,7 +10243,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A64" s="5" t="s">
         <v>259</v>
       </c>
@@ -10286,7 +10296,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A65" s="5" t="s">
         <v>262</v>
       </c>
@@ -10339,7 +10349,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A66" s="5" t="s">
         <v>269</v>
       </c>
@@ -10392,7 +10402,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A67" s="5" t="s">
         <v>275</v>
       </c>
@@ -10445,7 +10455,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A68" s="5" t="s">
         <v>282</v>
       </c>
@@ -10498,7 +10508,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A69" s="5" t="s">
         <v>285</v>
       </c>
@@ -10551,7 +10561,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A70" s="5" t="s">
         <v>289</v>
       </c>
@@ -10604,7 +10614,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A71" s="5" t="s">
         <v>295</v>
       </c>
@@ -10657,7 +10667,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A72" s="5" t="s">
         <v>300</v>
       </c>
@@ -10710,7 +10720,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A73" s="5" t="s">
         <v>307</v>
       </c>
@@ -10763,7 +10773,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A74" s="5" t="s">
         <v>309</v>
       </c>
@@ -10816,7 +10826,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:17" ht="64" x14ac:dyDescent="0.2">
       <c r="A75" s="5" t="s">
         <v>315</v>
       </c>
@@ -10869,7 +10879,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A76" s="5" t="s">
         <v>321</v>
       </c>
@@ -10922,7 +10932,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A77" s="5" t="s">
         <v>327</v>
       </c>
@@ -10975,7 +10985,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A78" s="5" t="s">
         <v>330</v>
       </c>
@@ -11028,7 +11038,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A79" s="5" t="s">
         <v>336</v>
       </c>
@@ -11081,7 +11091,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A80" s="5" t="s">
         <v>339</v>
       </c>
@@ -11134,7 +11144,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A81" s="5" t="s">
         <v>346</v>
       </c>
@@ -11187,7 +11197,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A82" s="5" t="s">
         <v>352</v>
       </c>
@@ -11240,7 +11250,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A83" s="5" t="s">
         <v>355</v>
       </c>
@@ -11293,7 +11303,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A84" s="5" t="s">
         <v>361</v>
       </c>
@@ -11346,7 +11356,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A85" s="5" t="s">
         <v>368</v>
       </c>
@@ -11399,7 +11409,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A86" s="5" t="s">
         <v>374</v>
       </c>
@@ -11452,7 +11462,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A87" s="5" t="s">
         <v>377</v>
       </c>
@@ -11505,7 +11515,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A88" s="5" t="s">
         <v>383</v>
       </c>
@@ -11558,7 +11568,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="89" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A89" s="5" t="s">
         <v>386</v>
       </c>
@@ -11611,7 +11621,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="90" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A90" s="5" t="s">
         <v>389</v>
       </c>
@@ -11664,7 +11674,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="91" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A91" s="5" t="s">
         <v>395</v>
       </c>
@@ -11717,7 +11727,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="92" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A92" s="5" t="s">
         <v>398</v>
       </c>
@@ -11770,7 +11780,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="93" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A93" s="5" t="s">
         <v>402</v>
       </c>
@@ -11823,7 +11833,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="94" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A94" s="5" t="s">
         <v>408</v>
       </c>
@@ -11876,7 +11886,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="95" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A95" s="5" t="s">
         <v>414</v>
       </c>
@@ -11929,7 +11939,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="96" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A96" s="5" t="s">
         <v>420</v>
       </c>
@@ -11964,7 +11974,7 @@
         <v>423</v>
       </c>
       <c r="L96" s="8" t="s">
-        <v>27</v>
+        <v>299</v>
       </c>
       <c r="M96" s="8" t="s">
         <v>26</v>
@@ -11982,7 +11992,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="97" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A97" s="5" t="s">
         <v>424</v>
       </c>
@@ -12035,7 +12045,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A98" s="5" t="s">
         <v>432</v>
       </c>
@@ -12088,7 +12098,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="99" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A99" s="5" t="s">
         <v>438</v>
       </c>
@@ -12141,7 +12151,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="100" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A100" s="5" t="s">
         <v>441</v>
       </c>
@@ -12194,7 +12204,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="101" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A101" s="5" t="s">
         <v>446</v>
       </c>
@@ -12247,7 +12257,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="102" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A102" s="5" t="s">
         <v>449</v>
       </c>
@@ -12300,7 +12310,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A103" s="5" t="s">
         <v>452</v>
       </c>
@@ -12353,7 +12363,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="104" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A104" s="5" t="s">
         <v>456</v>
       </c>
@@ -12406,7 +12416,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="105" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A105" s="5" t="s">
         <v>459</v>
       </c>
@@ -12459,7 +12469,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="106" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A106" s="5" t="s">
         <v>462</v>
       </c>
@@ -12512,7 +12522,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="107" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A107" s="5" t="s">
         <v>468</v>
       </c>
@@ -12565,7 +12575,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="108" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A108" s="5" t="s">
         <v>474</v>
       </c>
@@ -12618,7 +12628,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A109" s="5" t="s">
         <v>477</v>
       </c>
@@ -12671,7 +12681,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="110" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A110" s="5" t="s">
         <v>480</v>
       </c>
@@ -12724,7 +12734,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="111" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A111" s="5" t="s">
         <v>486</v>
       </c>
@@ -12777,7 +12787,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="112" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A112" s="5" t="s">
         <v>492</v>
       </c>
@@ -12830,7 +12840,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="113" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A113" s="5" t="s">
         <v>498</v>
       </c>
@@ -12883,7 +12893,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="114" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A114" s="5" t="s">
         <v>501</v>
       </c>
@@ -12936,7 +12946,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="115" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A115" s="5" t="s">
         <v>507</v>
       </c>
@@ -12989,7 +12999,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="116" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A116" s="5" t="s">
         <v>510</v>
       </c>
@@ -13042,7 +13052,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="117" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A117" s="5" t="s">
         <v>513</v>
       </c>
@@ -13095,7 +13105,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="118" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A118" s="5" t="s">
         <v>516</v>
       </c>
@@ -13148,7 +13158,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="119" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A119" s="5" t="s">
         <v>519</v>
       </c>
@@ -13201,7 +13211,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="120" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A120" s="5" t="s">
         <v>522</v>
       </c>
@@ -13254,7 +13264,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="121" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A121" s="5" t="s">
         <v>525</v>
       </c>
@@ -13307,7 +13317,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="122" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A122" s="5" t="s">
         <v>531</v>
       </c>
@@ -13360,7 +13370,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="123" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A123" s="5" t="s">
         <v>534</v>
       </c>
@@ -13413,7 +13423,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="124" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A124" s="5" t="s">
         <v>537</v>
       </c>
@@ -13466,7 +13476,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="125" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A125" s="5" t="s">
         <v>540</v>
       </c>
@@ -13519,7 +13529,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="126" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A126" s="5" t="s">
         <v>543</v>
       </c>
@@ -13572,7 +13582,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="127" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A127" s="5" t="s">
         <v>546</v>
       </c>
@@ -13625,7 +13635,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="128" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A128" s="5" t="s">
         <v>552</v>
       </c>
@@ -13678,7 +13688,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="129" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A129" s="5" t="s">
         <v>555</v>
       </c>
@@ -13731,7 +13741,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="130" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A130" s="5" t="s">
         <v>559</v>
       </c>
@@ -13784,7 +13794,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="131" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A131" s="5" t="s">
         <v>562</v>
       </c>
@@ -13837,7 +13847,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="132" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A132" s="5" t="s">
         <v>565</v>
       </c>
@@ -13890,7 +13900,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="133" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A133" s="5" t="s">
         <v>571</v>
       </c>
@@ -13943,7 +13953,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="134" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A134" s="5" t="s">
         <v>574</v>
       </c>
@@ -13996,7 +14006,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="135" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A135" s="5" t="s">
         <v>580</v>
       </c>
@@ -14049,7 +14059,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="136" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A136" s="5" t="s">
         <v>583</v>
       </c>
@@ -14102,7 +14112,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="137" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A137" s="5" t="s">
         <v>586</v>
       </c>
@@ -14155,7 +14165,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="138" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A138" s="5" t="s">
         <v>590</v>
       </c>
@@ -14208,7 +14218,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="139" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A139" s="5" t="s">
         <v>596</v>
       </c>
@@ -14261,7 +14271,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="140" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A140" s="5" t="s">
         <v>599</v>
       </c>
@@ -14314,7 +14324,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="141" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A141" s="5" t="s">
         <v>602</v>
       </c>
@@ -14367,7 +14377,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="142" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A142" s="5" t="s">
         <v>608</v>
       </c>
@@ -14420,7 +14430,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="143" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A143" s="5" t="s">
         <v>611</v>
       </c>
@@ -14473,7 +14483,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="144" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A144" s="5" t="s">
         <v>614</v>
       </c>
@@ -14526,7 +14536,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="145" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A145" s="5" t="s">
         <v>617</v>
       </c>
@@ -14579,7 +14589,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="146" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A146" s="5" t="s">
         <v>620</v>
       </c>
@@ -14632,7 +14642,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="147" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A147" s="5" t="s">
         <v>626</v>
       </c>
@@ -14685,7 +14695,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="148" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A148" s="5" t="s">
         <v>632</v>
       </c>
@@ -14738,7 +14748,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="149" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A149" s="5" t="s">
         <v>638</v>
       </c>
@@ -14791,7 +14801,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="150" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A150" s="5" t="s">
         <v>641</v>
       </c>
@@ -14844,7 +14854,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="151" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A151" s="5" t="s">
         <v>644</v>
       </c>
@@ -14897,7 +14907,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="152" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A152" s="5" t="s">
         <v>647</v>
       </c>
@@ -14950,7 +14960,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="153" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A153" s="5" t="s">
         <v>650</v>
       </c>
@@ -15003,7 +15013,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="154" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A154" s="5" t="s">
         <v>653</v>
       </c>
@@ -15056,7 +15066,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="155" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A155" s="5" t="s">
         <v>656</v>
       </c>
@@ -15109,7 +15119,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="156" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A156" s="5" t="s">
         <v>659</v>
       </c>
@@ -15162,7 +15172,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="157" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A157" s="5" t="s">
         <v>662</v>
       </c>
@@ -15215,7 +15225,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="158" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A158" s="5" t="s">
         <v>668</v>
       </c>
@@ -15268,7 +15278,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="159" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A159" s="5" t="s">
         <v>674</v>
       </c>
@@ -15321,7 +15331,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="160" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A160" s="5" t="s">
         <v>677</v>
       </c>
@@ -15374,7 +15384,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="161" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A161" s="5" t="s">
         <v>680</v>
       </c>
@@ -15427,7 +15437,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="162" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A162" s="5" t="s">
         <v>683</v>
       </c>
@@ -15480,7 +15490,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="163" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A163" s="5" t="s">
         <v>686</v>
       </c>
@@ -15533,7 +15543,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="164" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A164" s="5" t="s">
         <v>689</v>
       </c>
@@ -15586,7 +15596,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="165" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A165" s="5" t="s">
         <v>692</v>
       </c>
@@ -15639,7 +15649,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="166" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A166" s="5" t="s">
         <v>695</v>
       </c>
@@ -15692,7 +15702,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="167" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A167" s="5" t="s">
         <v>698</v>
       </c>
@@ -15745,7 +15755,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="168" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A168" s="5" t="s">
         <v>701</v>
       </c>
@@ -15798,7 +15808,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="169" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A169" s="5" t="s">
         <v>704</v>
       </c>
@@ -15851,7 +15861,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="170" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A170" s="5" t="s">
         <v>708</v>
       </c>
@@ -15904,7 +15914,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="171" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A171" s="5" t="s">
         <v>711</v>
       </c>
@@ -15957,7 +15967,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="172" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A172" s="5" t="s">
         <v>718</v>
       </c>
@@ -16010,7 +16020,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="173" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A173" s="5" t="s">
         <v>724</v>
       </c>
@@ -16063,7 +16073,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="174" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A174" s="5" t="s">
         <v>730</v>
       </c>
@@ -16116,7 +16126,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="175" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A175" s="5" t="s">
         <v>736</v>
       </c>
@@ -16169,7 +16179,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="176" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A176" s="5" t="s">
         <v>739</v>
       </c>
@@ -16222,7 +16232,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="177" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A177" s="5" t="s">
         <v>743</v>
       </c>
@@ -16275,7 +16285,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="178" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A178" s="5" t="s">
         <v>747</v>
       </c>
@@ -16328,7 +16338,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="179" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A179" s="5" t="s">
         <v>753</v>
       </c>
@@ -16381,7 +16391,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="180" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A180" s="5" t="s">
         <v>759</v>
       </c>
@@ -16434,7 +16444,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="181" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A181" s="5" t="s">
         <v>762</v>
       </c>
@@ -16487,7 +16497,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="182" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A182" s="5" t="s">
         <v>768</v>
       </c>
@@ -16540,7 +16550,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="183" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A183" s="5" t="s">
         <v>774</v>
       </c>
@@ -16593,7 +16603,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="184" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A184" s="5" t="s">
         <v>780</v>
       </c>
@@ -16646,7 +16656,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="185" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A185" s="5" t="s">
         <v>783</v>
       </c>
@@ -16699,7 +16709,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="186" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A186" s="5" t="s">
         <v>789</v>
       </c>
@@ -16752,7 +16762,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="187" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A187" s="5" t="s">
         <v>795</v>
       </c>
@@ -16805,7 +16815,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="188" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A188" s="5" t="s">
         <v>801</v>
       </c>
@@ -16858,7 +16868,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="189" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A189" s="5" t="s">
         <v>804</v>
       </c>
@@ -16911,7 +16921,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="190" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A190" s="5" t="s">
         <v>810</v>
       </c>
@@ -16964,7 +16974,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="191" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A191" s="5" t="s">
         <v>813</v>
       </c>
@@ -17017,7 +17027,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="192" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A192" s="5" t="s">
         <v>819</v>
       </c>
@@ -17070,7 +17080,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="193" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A193" s="5" t="s">
         <v>825</v>
       </c>
@@ -17123,7 +17133,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="194" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A194" s="5" t="s">
         <v>831</v>
       </c>
@@ -17176,7 +17186,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="195" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A195" s="5" t="s">
         <v>837</v>
       </c>
@@ -17229,7 +17239,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="196" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A196" s="5" t="s">
         <v>843</v>
       </c>
@@ -17282,7 +17292,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="197" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A197" s="5" t="s">
         <v>849</v>
       </c>
@@ -17335,7 +17345,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="198" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A198" s="5" t="s">
         <v>855</v>
       </c>
@@ -17388,7 +17398,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="199" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A199" s="5" t="s">
         <v>861</v>
       </c>
@@ -17441,7 +17451,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="200" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A200" s="5" t="s">
         <v>867</v>
       </c>
@@ -17494,7 +17504,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="201" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A201" s="5" t="s">
         <v>873</v>
       </c>
@@ -17547,7 +17557,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="202" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A202" s="5" t="s">
         <v>879</v>
       </c>
@@ -17600,7 +17610,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="203" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A203" s="5" t="s">
         <v>882</v>
       </c>
@@ -17653,7 +17663,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="204" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A204" s="5" t="s">
         <v>888</v>
       </c>
@@ -17706,7 +17716,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="205" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A205" s="5" t="s">
         <v>894</v>
       </c>
@@ -17759,7 +17769,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="206" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A206" s="5" t="s">
         <v>900</v>
       </c>
@@ -17812,7 +17822,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="207" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A207" s="5" t="s">
         <v>906</v>
       </c>
@@ -17865,7 +17875,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="208" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A208" s="5" t="s">
         <v>912</v>
       </c>
@@ -17918,7 +17928,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="209" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A209" s="5" t="s">
         <v>918</v>
       </c>
@@ -17971,7 +17981,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="210" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A210" s="5" t="s">
         <v>921</v>
       </c>
@@ -18024,7 +18034,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="211" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A211" s="5" t="s">
         <v>924</v>
       </c>
@@ -18077,7 +18087,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="212" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A212" s="5" t="s">
         <v>930</v>
       </c>
@@ -18130,7 +18140,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="213" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A213" s="5" t="s">
         <v>936</v>
       </c>
@@ -18183,7 +18193,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="214" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A214" s="5" t="s">
         <v>942</v>
       </c>
@@ -18236,7 +18246,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="215" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A215" s="5" t="s">
         <v>945</v>
       </c>
@@ -18289,7 +18299,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="216" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A216" s="5" t="s">
         <v>948</v>
       </c>
@@ -18342,7 +18352,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="217" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A217" s="5" t="s">
         <v>951</v>
       </c>
@@ -18395,7 +18405,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="218" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A218" s="5" t="s">
         <v>957</v>
       </c>
@@ -18448,7 +18458,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="219" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A219" s="5" t="s">
         <v>963</v>
       </c>
@@ -18501,7 +18511,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="220" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A220" s="5" t="s">
         <v>969</v>
       </c>
@@ -18554,7 +18564,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="221" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A221" s="5" t="s">
         <v>975</v>
       </c>
@@ -18607,7 +18617,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="222" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A222" s="5" t="s">
         <v>981</v>
       </c>
@@ -18660,7 +18670,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="223" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A223" s="5" t="s">
         <v>984</v>
       </c>
@@ -18713,7 +18723,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="224" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A224" s="5" t="s">
         <v>987</v>
       </c>
@@ -18766,7 +18776,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="225" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A225" s="5" t="s">
         <v>990</v>
       </c>
@@ -18819,7 +18829,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="226" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A226" s="5" t="s">
         <v>996</v>
       </c>
@@ -18872,7 +18882,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="227" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A227" s="5" t="s">
         <v>1002</v>
       </c>
@@ -18925,7 +18935,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="228" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A228" s="5" t="s">
         <v>1008</v>
       </c>
@@ -18978,7 +18988,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="229" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A229" s="5" t="s">
         <v>1014</v>
       </c>
@@ -19031,7 +19041,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="230" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A230" s="5" t="s">
         <v>1020</v>
       </c>
@@ -19084,7 +19094,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="231" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A231" s="5" t="s">
         <v>1026</v>
       </c>
@@ -19137,7 +19147,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="232" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A232" s="5" t="s">
         <v>1032</v>
       </c>
@@ -19190,7 +19200,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="233" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A233" s="5" t="s">
         <v>1035</v>
       </c>
@@ -19243,7 +19253,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="234" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A234" s="5" t="s">
         <v>1038</v>
       </c>
@@ -19296,7 +19306,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="235" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A235" s="5" t="s">
         <v>1044</v>
       </c>
@@ -19349,7 +19359,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="236" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A236" s="5" t="s">
         <v>1050</v>
       </c>
@@ -19402,7 +19412,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="237" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A237" s="5" t="s">
         <v>1056</v>
       </c>
@@ -19455,7 +19465,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="238" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A238" s="5" t="s">
         <v>1059</v>
       </c>
@@ -19508,7 +19518,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="239" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A239" s="5" t="s">
         <v>1062</v>
       </c>
@@ -19561,7 +19571,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="240" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A240" s="5" t="s">
         <v>1068</v>
       </c>
@@ -19614,7 +19624,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="241" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A241" s="5" t="s">
         <v>1074</v>
       </c>
@@ -19667,7 +19677,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="242" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A242" s="5" t="s">
         <v>1077</v>
       </c>
@@ -19720,7 +19730,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="243" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A243" s="5" t="s">
         <v>1080</v>
       </c>
@@ -19773,7 +19783,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="244" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A244" s="5" t="s">
         <v>1083</v>
       </c>
@@ -19826,7 +19836,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="245" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A245" s="5" t="s">
         <v>1086</v>
       </c>
@@ -19879,7 +19889,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="246" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A246" s="5" t="s">
         <v>1092</v>
       </c>
@@ -19932,7 +19942,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="247" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A247" s="5" t="s">
         <v>1098</v>
       </c>
@@ -19985,7 +19995,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="248" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A248" s="5" t="s">
         <v>1104</v>
       </c>
@@ -20038,7 +20048,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="249" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A249" s="5" t="s">
         <v>1110</v>
       </c>
@@ -20091,7 +20101,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="250" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A250" s="5" t="s">
         <v>1113</v>
       </c>
@@ -20144,7 +20154,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="251" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A251" s="5" t="s">
         <v>1116</v>
       </c>
@@ -20197,7 +20207,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="252" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A252" s="5" t="s">
         <v>1119</v>
       </c>
@@ -20250,7 +20260,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="253" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A253" s="5" t="s">
         <v>1125</v>
       </c>
@@ -20303,7 +20313,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="254" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A254" s="5" t="s">
         <v>1128</v>
       </c>
@@ -20356,7 +20366,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="255" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A255" s="5" t="s">
         <v>1131</v>
       </c>
@@ -20409,7 +20419,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="256" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A256" s="5" t="s">
         <v>1134</v>
       </c>
@@ -20462,7 +20472,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="257" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A257" s="5" t="s">
         <v>1140</v>
       </c>
@@ -20515,7 +20525,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="258" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A258" s="5" t="s">
         <v>1146</v>
       </c>
@@ -20568,7 +20578,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="259" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A259" s="5" t="s">
         <v>1149</v>
       </c>
@@ -20621,7 +20631,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="260" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A260" s="5" t="s">
         <v>1155</v>
       </c>
@@ -20674,7 +20684,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="261" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A261" s="5" t="s">
         <v>1161</v>
       </c>
@@ -20727,7 +20737,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="262" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A262" s="5" t="s">
         <v>1164</v>
       </c>
@@ -20780,7 +20790,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="263" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A263" s="5" t="s">
         <v>1170</v>
       </c>
@@ -20833,7 +20843,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="264" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A264" s="5" t="s">
         <v>1173</v>
       </c>
@@ -20886,7 +20896,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="265" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A265" s="5" t="s">
         <v>1179</v>
       </c>
@@ -20939,7 +20949,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="266" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A266" s="5" t="s">
         <v>1182</v>
       </c>
@@ -20992,7 +21002,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="267" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A267" s="5" t="s">
         <v>1185</v>
       </c>
@@ -21045,7 +21055,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="268" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A268" s="5" t="s">
         <v>1191</v>
       </c>
@@ -21098,7 +21108,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="269" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A269" s="5" t="s">
         <v>1194</v>
       </c>
@@ -21151,7 +21161,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="270" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A270" s="5" t="s">
         <v>1197</v>
       </c>
@@ -21204,7 +21214,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="271" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A271" s="5" t="s">
         <v>1200</v>
       </c>
@@ -21257,7 +21267,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="272" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A272" s="5" t="s">
         <v>1206</v>
       </c>
@@ -21310,7 +21320,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="273" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A273" s="5" t="s">
         <v>1209</v>
       </c>
@@ -21363,7 +21373,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="274" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A274" s="5" t="s">
         <v>1212</v>
       </c>
@@ -21416,7 +21426,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="275" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A275" s="5" t="s">
         <v>1218</v>
       </c>
@@ -21469,7 +21479,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="276" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A276" s="5" t="s">
         <v>1221</v>
       </c>
@@ -21522,7 +21532,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="277" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A277" s="5" t="s">
         <v>1224</v>
       </c>
@@ -21575,7 +21585,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="278" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A278" s="5" t="s">
         <v>1230</v>
       </c>
@@ -21628,7 +21638,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="279" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A279" s="5" t="s">
         <v>1234</v>
       </c>
@@ -21681,7 +21691,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="280" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A280" s="5" t="s">
         <v>1237</v>
       </c>
@@ -21734,7 +21744,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="281" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A281" s="5" t="s">
         <v>1240</v>
       </c>
@@ -21787,7 +21797,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="282" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A282" s="5" t="s">
         <v>1243</v>
       </c>
@@ -21840,7 +21850,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="283" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A283" s="5" t="s">
         <v>1249</v>
       </c>
@@ -21893,7 +21903,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="284" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A284" s="5" t="s">
         <v>1252</v>
       </c>
@@ -21946,7 +21956,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="285" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A285" s="5" t="s">
         <v>1255</v>
       </c>
@@ -21999,7 +22009,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="286" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A286" s="5" t="s">
         <v>1258</v>
       </c>
@@ -22052,7 +22062,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="287" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A287" s="5" t="s">
         <v>1261</v>
       </c>
@@ -22105,7 +22115,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="288" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A288" s="5" t="s">
         <v>1264</v>
       </c>
@@ -22158,7 +22168,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="289" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A289" s="5" t="s">
         <v>1267</v>
       </c>
@@ -22211,7 +22221,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="290" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A290" s="5" t="s">
         <v>1270</v>
       </c>
@@ -22264,7 +22274,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="291" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A291" s="5" t="s">
         <v>1276</v>
       </c>
@@ -22317,7 +22327,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="292" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A292" s="5" t="s">
         <v>1279</v>
       </c>
@@ -22370,7 +22380,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="293" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A293" s="5" t="s">
         <v>1285</v>
       </c>
@@ -22423,7 +22433,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="294" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A294" s="5" t="s">
         <v>1291</v>
       </c>
@@ -22476,7 +22486,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="295" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A295" s="5" t="s">
         <v>1294</v>
       </c>
@@ -22529,7 +22539,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="296" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A296" s="5" t="s">
         <v>1300</v>
       </c>
@@ -22582,7 +22592,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="297" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A297" s="5" t="s">
         <v>1303</v>
       </c>
@@ -22635,7 +22645,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="298" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A298" s="5" t="s">
         <v>1306</v>
       </c>
@@ -22688,7 +22698,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="299" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A299" s="5" t="s">
         <v>1309</v>
       </c>
@@ -22741,7 +22751,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="300" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A300" s="5" t="s">
         <v>1312</v>
       </c>
@@ -22794,7 +22804,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="301" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A301" s="5" t="s">
         <v>1315</v>
       </c>
@@ -22847,7 +22857,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="302" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A302" s="5" t="s">
         <v>1321</v>
       </c>
@@ -22900,7 +22910,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="303" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A303" s="5" t="s">
         <v>1324</v>
       </c>
@@ -22953,7 +22963,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="304" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A304" s="5" t="s">
         <v>1330</v>
       </c>
@@ -23006,7 +23016,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="305" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A305" s="5" t="s">
         <v>1333</v>
       </c>
@@ -23059,7 +23069,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="306" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A306" s="5" t="s">
         <v>1339</v>
       </c>
@@ -23112,7 +23122,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="307" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A307" s="5" t="s">
         <v>1345</v>
       </c>
@@ -23165,7 +23175,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="308" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A308" s="5" t="s">
         <v>1348</v>
       </c>
@@ -23218,7 +23228,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="309" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A309" s="5" t="s">
         <v>1351</v>
       </c>
@@ -23271,7 +23281,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="310" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A310" s="5" t="s">
         <v>1354</v>
       </c>
@@ -23324,7 +23334,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="311" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A311" s="5" t="s">
         <v>1360</v>
       </c>
@@ -23377,7 +23387,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="312" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A312" s="5" t="s">
         <v>1363</v>
       </c>
@@ -23430,7 +23440,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="313" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A313" s="5" t="s">
         <v>1369</v>
       </c>
@@ -23483,7 +23493,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="314" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A314" s="5" t="s">
         <v>1373</v>
       </c>
@@ -23536,7 +23546,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="315" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A315" s="5" t="s">
         <v>1375</v>
       </c>
@@ -23589,7 +23599,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="316" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A316" s="5" t="s">
         <v>1381</v>
       </c>
@@ -23642,7 +23652,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="317" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A317" s="5" t="s">
         <v>1387</v>
       </c>
@@ -23695,7 +23705,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="318" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A318" s="5" t="s">
         <v>1393</v>
       </c>
@@ -23748,7 +23758,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="319" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A319" s="5" t="s">
         <v>1399</v>
       </c>
@@ -23801,7 +23811,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="320" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A320" s="5" t="s">
         <v>1405</v>
       </c>
@@ -23854,7 +23864,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="321" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A321" s="5" t="s">
         <v>1408</v>
       </c>
@@ -23907,7 +23917,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="322" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A322" s="5" t="s">
         <v>1414</v>
       </c>
@@ -23960,7 +23970,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="323" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A323" s="5" t="s">
         <v>1417</v>
       </c>
@@ -24013,7 +24023,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="324" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A324" s="5" t="s">
         <v>1423</v>
       </c>
@@ -24066,7 +24076,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="325" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A325" s="5" t="s">
         <v>1429</v>
       </c>
@@ -24119,7 +24129,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="326" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A326" s="5" t="s">
         <v>1432</v>
       </c>
@@ -24172,7 +24182,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="327" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A327" s="5" t="s">
         <v>1438</v>
       </c>
@@ -24225,7 +24235,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="328" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A328" s="5" t="s">
         <v>1444</v>
       </c>
@@ -24278,7 +24288,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="329" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A329" s="5" t="s">
         <v>1450</v>
       </c>
@@ -24331,7 +24341,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="330" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A330" s="5" t="s">
         <v>1453</v>
       </c>
@@ -24384,7 +24394,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="331" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A331" s="5" t="s">
         <v>1456</v>
       </c>
@@ -24437,7 +24447,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="332" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A332" s="5" t="s">
         <v>1459</v>
       </c>
@@ -24490,7 +24500,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="333" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A333" s="5" t="s">
         <v>1465</v>
       </c>
@@ -24543,7 +24553,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="334" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A334" s="5" t="s">
         <v>1468</v>
       </c>
@@ -24596,7 +24606,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="335" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A335" s="5" t="s">
         <v>1474</v>
       </c>
@@ -24649,7 +24659,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="336" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A336" s="5" t="s">
         <v>1477</v>
       </c>
@@ -24702,7 +24712,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="337" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A337" s="5" t="s">
         <v>1483</v>
       </c>
@@ -24755,7 +24765,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="338" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A338" s="5" t="s">
         <v>1486</v>
       </c>
@@ -24808,7 +24818,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="339" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A339" s="5" t="s">
         <v>1492</v>
       </c>
@@ -24861,7 +24871,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="340" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A340" s="5" t="s">
         <v>1498</v>
       </c>
@@ -24914,7 +24924,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="341" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A341" s="5" t="s">
         <v>1501</v>
       </c>
@@ -24967,7 +24977,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="342" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A342" s="5" t="s">
         <v>1504</v>
       </c>
@@ -25020,7 +25030,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="343" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A343" s="5" t="s">
         <v>1507</v>
       </c>
@@ -25073,7 +25083,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="344" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A344" s="5" t="s">
         <v>1511</v>
       </c>
@@ -25126,7 +25136,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="345" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A345" s="5" t="s">
         <v>1514</v>
       </c>
@@ -25179,7 +25189,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="346" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A346" s="5" t="s">
         <v>1517</v>
       </c>
@@ -25232,7 +25242,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="347" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A347" s="5" t="s">
         <v>1520</v>
       </c>
@@ -25285,7 +25295,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="348" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A348" s="5" t="s">
         <v>1526</v>
       </c>
@@ -25338,7 +25348,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="349" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A349" s="5" t="s">
         <v>1529</v>
       </c>
@@ -25391,7 +25401,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="350" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A350" s="5" t="s">
         <v>1532</v>
       </c>
@@ -25444,7 +25454,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="351" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A351" s="5" t="s">
         <v>1538</v>
       </c>
@@ -25497,7 +25507,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="352" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A352" s="5" t="s">
         <v>1541</v>
       </c>
@@ -25550,7 +25560,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="353" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A353" s="5" t="s">
         <v>1544</v>
       </c>
@@ -25603,7 +25613,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="354" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A354" s="5" t="s">
         <v>1547</v>
       </c>
@@ -25656,7 +25666,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="355" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A355" s="5" t="s">
         <v>1553</v>
       </c>
@@ -25709,7 +25719,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="356" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A356" s="5" t="s">
         <v>1556</v>
       </c>
@@ -25762,7 +25772,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="357" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A357" s="5" t="s">
         <v>1559</v>
       </c>
@@ -25815,7 +25825,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="358" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A358" s="5" t="s">
         <v>1562</v>
       </c>
@@ -25868,7 +25878,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="359" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A359" s="5" t="s">
         <v>1568</v>
       </c>
@@ -25921,7 +25931,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="360" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A360" s="5" t="s">
         <v>1574</v>
       </c>
@@ -25974,7 +25984,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="361" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A361" s="5" t="s">
         <v>1577</v>
       </c>
@@ -26027,7 +26037,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="362" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A362" s="5" t="s">
         <v>1580</v>
       </c>
@@ -26080,7 +26090,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="363" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A363" s="5" t="s">
         <v>1586</v>
       </c>
@@ -26133,7 +26143,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="364" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A364" s="5" t="s">
         <v>1589</v>
       </c>
@@ -26186,7 +26196,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="365" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A365" s="5" t="s">
         <v>1592</v>
       </c>
@@ -26239,7 +26249,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="366" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A366" s="5" t="s">
         <v>1595</v>
       </c>
@@ -26292,7 +26302,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="367" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A367" s="5" t="s">
         <v>1601</v>
       </c>
@@ -26345,7 +26355,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="368" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A368" s="5" t="s">
         <v>1604</v>
       </c>
@@ -26398,7 +26408,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="369" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A369" s="5" t="s">
         <v>1610</v>
       </c>
@@ -26451,7 +26461,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="370" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A370" s="5" t="s">
         <v>1613</v>
       </c>
@@ -26504,7 +26514,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="371" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A371" s="5" t="s">
         <v>1616</v>
       </c>
@@ -26557,7 +26567,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="372" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A372" s="5" t="s">
         <v>1619</v>
       </c>
@@ -26610,7 +26620,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="373" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A373" s="5" t="s">
         <v>1622</v>
       </c>
@@ -26663,7 +26673,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="374" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A374" s="5" t="s">
         <v>1625</v>
       </c>
@@ -26716,7 +26726,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="375" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A375" s="5" t="s">
         <v>1628</v>
       </c>
@@ -26769,7 +26779,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="376" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A376" s="5" t="s">
         <v>1631</v>
       </c>
@@ -26822,7 +26832,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="377" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A377" s="5" t="s">
         <v>1634</v>
       </c>
@@ -26875,7 +26885,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="378" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A378" s="5" t="s">
         <v>1637</v>
       </c>
@@ -26928,7 +26938,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="379" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A379" s="5" t="s">
         <v>1643</v>
       </c>
@@ -26981,7 +26991,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="380" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A380" s="5" t="s">
         <v>1646</v>
       </c>
@@ -27034,7 +27044,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="381" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A381" s="5" t="s">
         <v>1649</v>
       </c>
@@ -27087,7 +27097,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="382" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A382" s="5" t="s">
         <v>1652</v>
       </c>
@@ -27140,7 +27150,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="383" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A383" s="5" t="s">
         <v>1658</v>
       </c>
@@ -27193,7 +27203,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="384" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A384" s="5" t="s">
         <v>1661</v>
       </c>
@@ -27246,7 +27256,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="385" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A385" s="5" t="s">
         <v>1667</v>
       </c>
@@ -27299,7 +27309,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="386" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A386" s="5" t="s">
         <v>1670</v>
       </c>
@@ -27352,7 +27362,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="387" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A387" s="5" t="s">
         <v>1673</v>
       </c>
@@ -27405,7 +27415,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="388" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A388" s="5" t="s">
         <v>1676</v>
       </c>
@@ -27458,7 +27468,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="389" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A389" s="5" t="s">
         <v>1679</v>
       </c>
@@ -27511,7 +27521,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="390" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A390" s="5" t="s">
         <v>1682</v>
       </c>
@@ -27564,7 +27574,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="391" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A391" s="5" t="s">
         <v>1688</v>
       </c>
@@ -27617,7 +27627,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="392" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A392" s="5" t="s">
         <v>1694</v>
       </c>
@@ -27670,7 +27680,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="393" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A393" s="5" t="s">
         <v>1697</v>
       </c>
@@ -27723,7 +27733,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="394" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A394" s="5" t="s">
         <v>1700</v>
       </c>
@@ -27776,7 +27786,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="395" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A395" s="5" t="s">
         <v>1707</v>
       </c>
@@ -27829,7 +27839,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="396" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A396" s="5" t="s">
         <v>1709</v>
       </c>
@@ -27882,7 +27892,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="397" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A397" s="5" t="s">
         <v>1712</v>
       </c>
@@ -27935,7 +27945,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="398" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A398" s="5" t="s">
         <v>1715</v>
       </c>
@@ -27988,7 +27998,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="399" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A399" s="5" t="s">
         <v>1721</v>
       </c>
@@ -28041,7 +28051,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="400" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A400" s="5" t="s">
         <v>1727</v>
       </c>
@@ -28094,7 +28104,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="401" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A401" s="5" t="s">
         <v>1730</v>
       </c>
@@ -28147,7 +28157,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="402" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A402" s="5" t="s">
         <v>1733</v>
       </c>
@@ -28200,7 +28210,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="403" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A403" s="5" t="s">
         <v>1736</v>
       </c>
@@ -28253,7 +28263,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="404" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A404" s="5" t="s">
         <v>1739</v>
       </c>
@@ -28306,7 +28316,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="405" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A405" s="5" t="s">
         <v>1742</v>
       </c>
@@ -28359,7 +28369,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="406" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A406" s="5" t="s">
         <v>1745</v>
       </c>
@@ -28412,7 +28422,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="407" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A407" s="5" t="s">
         <v>1751</v>
       </c>
@@ -28465,7 +28475,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="408" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A408" s="5" t="s">
         <v>1754</v>
       </c>
@@ -28518,7 +28528,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="409" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A409" s="5" t="s">
         <v>1757</v>
       </c>
@@ -28571,7 +28581,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="410" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="410" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A410" s="5" t="s">
         <v>1760</v>
       </c>
@@ -28624,7 +28634,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="411" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A411" s="5" t="s">
         <v>1763</v>
       </c>
@@ -28677,7 +28687,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="412" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A412" s="5" t="s">
         <v>1766</v>
       </c>
@@ -28730,7 +28740,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="413" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A413" s="5" t="s">
         <v>1772</v>
       </c>
@@ -28783,7 +28793,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="414" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A414" s="5" t="s">
         <v>1775</v>
       </c>
@@ -28836,7 +28846,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="415" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A415" s="5" t="s">
         <v>1781</v>
       </c>
@@ -28889,7 +28899,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="416" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="416" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A416" s="5" t="s">
         <v>1784</v>
       </c>
@@ -28942,7 +28952,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="417" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="417" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A417" s="5" t="s">
         <v>1790</v>
       </c>
@@ -28995,7 +29005,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="418" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A418" s="5" t="s">
         <v>1793</v>
       </c>
@@ -29048,7 +29058,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="419" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="419" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A419" s="5" t="s">
         <v>1796</v>
       </c>
@@ -29101,7 +29111,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="420" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="420" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A420" s="5" t="s">
         <v>1802</v>
       </c>
@@ -29154,7 +29164,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="421" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="421" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A421" s="5" t="s">
         <v>1805</v>
       </c>
@@ -29207,7 +29217,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="422" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="422" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A422" s="5" t="s">
         <v>1808</v>
       </c>
@@ -29260,7 +29270,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="423" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="423" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A423" s="5" t="s">
         <v>1811</v>
       </c>
@@ -29313,7 +29323,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="424" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="424" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A424" s="5" t="s">
         <v>1814</v>
       </c>
@@ -29366,7 +29376,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="425" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="425" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A425" s="5" t="s">
         <v>1817</v>
       </c>
@@ -29419,7 +29429,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="426" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="426" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A426" s="5" t="s">
         <v>1820</v>
       </c>
@@ -29472,7 +29482,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="427" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="427" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A427" s="5" t="s">
         <v>1823</v>
       </c>
@@ -29525,7 +29535,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="428" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="428" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A428" s="5" t="s">
         <v>1826</v>
       </c>
@@ -29578,7 +29588,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="429" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="429" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A429" s="5" t="s">
         <v>1829</v>
       </c>
@@ -29631,7 +29641,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="430" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="430" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A430" s="5" t="s">
         <v>1832</v>
       </c>
@@ -29684,7 +29694,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="431" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="431" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A431" s="5" t="s">
         <v>1838</v>
       </c>
@@ -29737,7 +29747,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="432" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="432" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A432" s="5" t="s">
         <v>1841</v>
       </c>
@@ -29790,7 +29800,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="433" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="433" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A433" s="5" t="s">
         <v>1844</v>
       </c>
@@ -29843,7 +29853,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="434" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="434" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A434" s="5" t="s">
         <v>1850</v>
       </c>
@@ -29896,7 +29906,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="435" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="435" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A435" s="5" t="s">
         <v>1856</v>
       </c>
@@ -29949,7 +29959,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="436" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="436" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A436" s="5" t="s">
         <v>1859</v>
       </c>
@@ -30002,7 +30012,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="437" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="437" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A437" s="5" t="s">
         <v>1862</v>
       </c>
@@ -30055,7 +30065,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="438" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="438" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A438" s="5" t="s">
         <v>1865</v>
       </c>
@@ -30108,7 +30118,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="439" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="439" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A439" s="5" t="s">
         <v>1868</v>
       </c>
@@ -30161,7 +30171,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="440" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="440" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A440" s="5" t="s">
         <v>1874</v>
       </c>
@@ -30214,7 +30224,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="441" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="441" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A441" s="5" t="s">
         <v>1877</v>
       </c>
@@ -30267,7 +30277,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="442" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="442" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A442" s="5" t="s">
         <v>1880</v>
       </c>
@@ -30320,7 +30330,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="443" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="443" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A443" s="5" t="s">
         <v>1883</v>
       </c>
@@ -30373,7 +30383,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="444" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="444" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A444" s="5" t="s">
         <v>1886</v>
       </c>
@@ -30426,7 +30436,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="445" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="445" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A445" s="5" t="s">
         <v>1889</v>
       </c>
@@ -30479,7 +30489,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="446" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="446" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A446" s="5" t="s">
         <v>1895</v>
       </c>
@@ -30532,7 +30542,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="447" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="447" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A447" s="5" t="s">
         <v>1898</v>
       </c>
@@ -30585,7 +30595,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="448" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="448" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A448" s="5" t="s">
         <v>1901</v>
       </c>
@@ -30638,7 +30648,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="449" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="449" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A449" s="5" t="s">
         <v>1904</v>
       </c>
@@ -30691,7 +30701,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="450" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="450" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A450" s="5" t="s">
         <v>1907</v>
       </c>
@@ -30744,7 +30754,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="451" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="451" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A451" s="5" t="s">
         <v>1910</v>
       </c>
@@ -30797,7 +30807,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="452" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="452" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A452" s="5" t="s">
         <v>1913</v>
       </c>
@@ -30850,7 +30860,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="453" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="453" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A453" s="5" t="s">
         <v>1916</v>
       </c>
@@ -30903,7 +30913,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="454" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="454" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A454" s="5" t="s">
         <v>1919</v>
       </c>
@@ -30956,7 +30966,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="455" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="455" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A455" s="5" t="s">
         <v>1925</v>
       </c>
@@ -31009,7 +31019,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="456" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="456" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A456" s="5" t="s">
         <v>1928</v>
       </c>
@@ -31062,7 +31072,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="457" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="457" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A457" s="5" t="s">
         <v>1934</v>
       </c>
@@ -31115,7 +31125,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="458" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="458" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A458" s="5" t="s">
         <v>1940</v>
       </c>
@@ -31168,7 +31178,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="459" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="459" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A459" s="5" t="s">
         <v>1943</v>
       </c>
@@ -31221,7 +31231,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="460" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="460" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A460" s="5" t="s">
         <v>1946</v>
       </c>
@@ -31274,7 +31284,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="461" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="461" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A461" s="5" t="s">
         <v>1952</v>
       </c>
@@ -31327,7 +31337,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="462" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="462" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A462" s="5" t="s">
         <v>1958</v>
       </c>
@@ -31380,7 +31390,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="463" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="463" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A463" s="5" t="s">
         <v>1964</v>
       </c>
@@ -31433,7 +31443,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="464" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="464" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A464" s="5" t="s">
         <v>1967</v>
       </c>
@@ -31486,7 +31496,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="465" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="465" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A465" s="5" t="s">
         <v>1970</v>
       </c>
@@ -31539,7 +31549,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="466" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="466" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A466" s="5" t="s">
         <v>1973</v>
       </c>
@@ -31592,7 +31602,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="467" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="467" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A467" s="5" t="s">
         <v>1976</v>
       </c>
@@ -31645,7 +31655,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="468" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="468" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A468" s="5" t="s">
         <v>1982</v>
       </c>
@@ -31698,7 +31708,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="469" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="469" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A469" s="5" t="s">
         <v>1985</v>
       </c>
@@ -31751,7 +31761,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="470" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="470" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A470" s="5" t="s">
         <v>1988</v>
       </c>
@@ -31804,7 +31814,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="471" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="471" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A471" s="5" t="s">
         <v>1991</v>
       </c>
@@ -31857,7 +31867,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="472" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="472" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A472" s="5" t="s">
         <v>1994</v>
       </c>
@@ -31910,7 +31920,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="473" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="473" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A473" s="5" t="s">
         <v>1997</v>
       </c>
@@ -31963,7 +31973,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="474" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="474" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A474" s="5" t="s">
         <v>2000</v>
       </c>
@@ -32016,7 +32026,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="475" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="475" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A475" s="5" t="s">
         <v>2006</v>
       </c>
@@ -32069,7 +32079,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="476" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="476" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A476" s="5" t="s">
         <v>2009</v>
       </c>
@@ -32122,7 +32132,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="477" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="477" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A477" s="5" t="s">
         <v>2015</v>
       </c>
@@ -32175,7 +32185,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="478" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="478" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A478" s="5" t="s">
         <v>2021</v>
       </c>
@@ -32228,7 +32238,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="479" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="479" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A479" s="5" t="s">
         <v>2024</v>
       </c>
@@ -32281,7 +32291,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="480" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="480" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A480" s="5" t="s">
         <v>2027</v>
       </c>
@@ -32334,7 +32344,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="481" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="481" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A481" s="5" t="s">
         <v>2030</v>
       </c>
@@ -32387,7 +32397,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="482" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="482" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A482" s="5" t="s">
         <v>2033</v>
       </c>
@@ -32440,7 +32450,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="483" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="483" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A483" s="5" t="s">
         <v>2036</v>
       </c>
@@ -32493,7 +32503,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="484" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="484" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A484" s="5" t="s">
         <v>2039</v>
       </c>
@@ -32546,7 +32556,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="485" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="485" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A485" s="5" t="s">
         <v>2045</v>
       </c>
@@ -32599,7 +32609,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="486" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="486" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A486" s="5" t="s">
         <v>2048</v>
       </c>
@@ -32652,7 +32662,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="487" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="487" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A487" s="5" t="s">
         <v>2051</v>
       </c>
@@ -32705,7 +32715,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="488" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="488" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A488" s="5" t="s">
         <v>2054</v>
       </c>
@@ -32758,7 +32768,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="489" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="489" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A489" s="5" t="s">
         <v>2057</v>
       </c>
@@ -32811,7 +32821,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="490" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="490" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A490" s="5" t="s">
         <v>2063</v>
       </c>
@@ -32864,7 +32874,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="491" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="491" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A491" s="5" t="s">
         <v>2066</v>
       </c>
@@ -32917,7 +32927,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="492" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="492" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A492" s="5" t="s">
         <v>2069</v>
       </c>
@@ -32970,7 +32980,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="493" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="493" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A493" s="5" t="s">
         <v>2072</v>
       </c>
@@ -33023,7 +33033,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="494" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="494" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A494" s="5" t="s">
         <v>2075</v>
       </c>
@@ -33076,7 +33086,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="495" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="495" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A495" s="5" t="s">
         <v>2078</v>
       </c>
@@ -33129,7 +33139,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="496" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="496" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A496" s="5" t="s">
         <v>2081</v>
       </c>
@@ -33182,7 +33192,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="497" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="497" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A497" s="5" t="s">
         <v>2087</v>
       </c>
@@ -33235,7 +33245,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="498" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="498" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A498" s="5" t="s">
         <v>2090</v>
       </c>
@@ -33288,7 +33298,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="499" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="499" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A499" s="5" t="s">
         <v>2093</v>
       </c>
@@ -33341,7 +33351,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="500" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="500" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A500" s="5" t="s">
         <v>2096</v>
       </c>
@@ -33394,7 +33404,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="501" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="501" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A501" s="5" t="s">
         <v>2099</v>
       </c>
@@ -33447,7 +33457,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="502" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="502" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A502" s="5" t="s">
         <v>2102</v>
       </c>
@@ -33500,7 +33510,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="503" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="503" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A503" s="5" t="s">
         <v>2105</v>
       </c>
@@ -33553,7 +33563,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="504" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="504" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A504" s="5" t="s">
         <v>2108</v>
       </c>
@@ -33606,7 +33616,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="505" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="505" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A505" s="5" t="s">
         <v>2113</v>
       </c>
@@ -33660,33 +33670,33 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q505"/>
+  <autoFilter ref="A1:Q505" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" prompt="ja = bleibt im Universum, nein = herausnehmen (z. B. delistet)" showErrorMessage="1" errorTitle="Ungültiger Wert" error="Erlaubt: ja, nein oder leer" sqref="L2:L505">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ungültiger Wert" error="Erlaubt: ja, nein oder leer" prompt="ja = bleibt im Universum, nein = herausnehmen (z. B. delistet)" sqref="L2:L505" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"ja,nein"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" prompt="Nur bei Börsenwechsel" showErrorMessage="1" errorTitle="Ungültiger Wert" error="Erlaubt: NYSE, NASDAQ, CBOE oder leer" sqref="O2:O505">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ungültiger Wert" error="Erlaubt: NYSE, NASDAQ, CBOE oder leer" prompt="Nur bei Börsenwechsel" sqref="O2:O505" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"NYSE,NASDAQ,CBOE"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" prompt="Nur ausfüllen, wenn die Behandlung abweichen soll. Begründung ist dann Pflicht." showErrorMessage="1" errorTitle="Ungültiger Wert" error="Erlaubt: exclude, review, b3_focus, allow oder leer" sqref="P2:P505">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ungültiger Wert" error="Erlaubt: exclude, review, b3_focus, allow oder leer" prompt="Nur ausfüllen, wenn die Behandlung abweichen soll. Begründung ist dann Pflicht." sqref="P2:P505" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"exclude,review,b3_focus,allow"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B26"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="10" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
         <v>2117</v>
       </c>
@@ -33694,7 +33704,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
         <v>24</v>
       </c>
@@ -33702,7 +33712,7 @@
         <v>2118</v>
       </c>
     </row>
-    <row r="3" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
         <v>267</v>
       </c>
@@ -33710,7 +33720,7 @@
         <v>2119</v>
       </c>
     </row>
-    <row r="4" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
         <v>430</v>
       </c>
@@ -33718,7 +33728,7 @@
         <v>2120</v>
       </c>
     </row>
-    <row r="5" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
         <v>716</v>
       </c>
@@ -33726,7 +33736,7 @@
         <v>2121</v>
       </c>
     </row>
-    <row r="6" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
         <v>2110</v>
       </c>
@@ -33734,7 +33744,7 @@
         <v>2122</v>
       </c>
     </row>
-    <row r="7" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
         <v>2115</v>
       </c>
@@ -33742,7 +33752,7 @@
         <v>2123</v>
       </c>
     </row>
-    <row r="8" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
         <v>26</v>
       </c>
@@ -33750,7 +33760,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:2" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" s="10" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="10" t="s">
         <v>2124</v>
       </c>
@@ -33758,7 +33768,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
         <v>2125</v>
       </c>
@@ -33766,7 +33776,7 @@
         <v>2126</v>
       </c>
     </row>
-    <row r="11" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
         <v>2</v>
       </c>
@@ -33774,7 +33784,7 @@
         <v>2127</v>
       </c>
     </row>
-    <row r="12" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
         <v>3</v>
       </c>
@@ -33782,7 +33792,7 @@
         <v>2128</v>
       </c>
     </row>
-    <row r="13" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
         <v>2129</v>
       </c>
@@ -33790,7 +33800,7 @@
         <v>2130</v>
       </c>
     </row>
-    <row r="14" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
         <v>6</v>
       </c>
@@ -33798,7 +33808,7 @@
         <v>2131</v>
       </c>
     </row>
-    <row r="15" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
         <v>7</v>
       </c>
@@ -33806,7 +33816,7 @@
         <v>2132</v>
       </c>
     </row>
-    <row r="16" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
         <v>8</v>
       </c>
@@ -33814,7 +33824,7 @@
         <v>2133</v>
       </c>
     </row>
-    <row r="17" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
         <v>9</v>
       </c>
@@ -33822,7 +33832,7 @@
         <v>2134</v>
       </c>
     </row>
-    <row r="18" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="11" t="s">
         <v>10</v>
       </c>
@@ -33830,7 +33840,7 @@
         <v>2135</v>
       </c>
     </row>
-    <row r="19" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="11" t="s">
         <v>26</v>
       </c>
@@ -33838,7 +33848,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:2" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" s="10" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A20" s="10" t="s">
         <v>2136</v>
       </c>
@@ -33846,7 +33856,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="21" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" s="11" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
         <v>11</v>
       </c>
@@ -33854,7 +33864,7 @@
         <v>2137</v>
       </c>
     </row>
-    <row r="22" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" s="11" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A22" s="11" t="s">
         <v>2138</v>
       </c>
@@ -33862,7 +33872,7 @@
         <v>2139</v>
       </c>
     </row>
-    <row r="23" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="11" t="s">
         <v>15</v>
       </c>
@@ -33870,7 +33880,7 @@
         <v>2140</v>
       </c>
     </row>
-    <row r="24" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="11" t="s">
         <v>16</v>
       </c>
@@ -33878,7 +33888,7 @@
         <v>2141</v>
       </c>
     </row>
-    <row r="25" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
         <v>26</v>
       </c>
@@ -33886,7 +33896,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" s="11" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A26" s="11" t="s">
         <v>2142</v>
       </c>
@@ -33896,6 +33906,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>